<commit_message>
data(W29): refresh WM other_channels — 1P Sales (9 rows)
Operator's manual 1P sales fill for WM (SP-API vendor blocked
per reference_wm_vendor_sp_api_blocked).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 29/White_Mulberry/other_channels.xlsx
+++ b/data/raw/sales/Week 29/White_Mulberry/other_channels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 29\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96B9995-D437-4E46-A720-0EF1B8B04C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CDBC59-A3B7-46CD-B994-3BF779090F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
   <si>
     <t>ASIN</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>White Mulberry</t>
+  </si>
+  <si>
+    <t>IN</t>
   </si>
 </sst>
 </file>
@@ -352,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C982260-665D-4839-80CC-B01F070D9895}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
@@ -362,7 +365,7 @@
     <col min="5" max="5" width="3.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -379,7 +382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -389,14 +392,29 @@
       <c r="C2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="1">
-        <v>74538.91</v>
-      </c>
-      <c r="E2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1">
+        <v>89785.52</v>
+      </c>
+      <c r="F2">
+        <v>53</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>54</v>
+      </c>
+      <c r="J2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -406,14 +424,29 @@
       <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1">
-        <v>30285.58</v>
-      </c>
-      <c r="E3">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="1">
+        <v>41933.879999999997</v>
+      </c>
+      <c r="F3">
+        <v>18</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>27</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -423,14 +456,29 @@
       <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="1">
-        <v>18325.939999999999</v>
-      </c>
-      <c r="E4">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1">
+        <v>31457.32</v>
+      </c>
+      <c r="F4">
+        <v>12</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>15</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -440,14 +488,29 @@
       <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1">
-        <v>10164.41</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="1">
+        <v>22022.9</v>
+      </c>
+      <c r="F5">
+        <v>13</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>13</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -457,14 +520,29 @@
       <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1">
-        <v>3643.22</v>
-      </c>
-      <c r="E6">
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="1">
+        <v>7286.44</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -474,45 +552,87 @@
       <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="1">
-        <v>2794.92</v>
-      </c>
-      <c r="E7">
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="1">
+        <v>4192.38</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1">
+        <v>288.13</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="1">
-        <v>-2414.41</v>
-      </c>
-      <c r="E9">
-        <v>-1</v>
+      <c r="J9">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>